<commit_message>
uporzadkowano komentarze, zmieniono formatowanie, zmieniono jezyk outputu na angielski
</commit_message>
<xml_diff>
--- a/zadanie_8/wyniki_z_wykresami.xlsx
+++ b/zadanie_8/wyniki_z_wykresami.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\barto\source\repos\Project62\Project62\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kołchoz\Algorytmy\Zadania\zadanie_8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AB774E72-2CC2-4E8D-A590-6059458A6475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C052D427-07C9-4F23-81B6-020A94446E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19545" windowHeight="15585" xr2:uid="{90626785-64BE-41CA-9FCD-EDCBB815A823}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{90626785-64BE-41CA-9FCD-EDCBB815A823}"/>
   </bookViews>
   <sheets>
     <sheet name="wyniki" sheetId="1" r:id="rId1"/>
@@ -710,12 +710,12 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent1"/>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="90000"/>
+                </a:schemeClr>
               </a:solidFill>
               <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
+                <a:noFill/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
@@ -7086,16 +7086,16 @@
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>1,758843</c:v>
+                  <c:v>1.758843</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1,681728</c:v>
+                  <c:v>1.681728</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1,592302</c:v>
+                  <c:v>1.592302</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1,368666</c:v>
+                  <c:v>1.368666</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -7447,11 +7447,13 @@
             <c:symbol val="circle"/>
             <c:size val="5"/>
             <c:spPr>
-              <a:noFill/>
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="90000"/>
+                </a:schemeClr>
+              </a:solidFill>
               <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
+                <a:noFill/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
@@ -8098,13 +8100,9 @@
             <c:symbol val="circle"/>
             <c:size val="5"/>
             <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="FF0000"/>
-              </a:solidFill>
+              <a:noFill/>
               <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent3"/>
-                </a:solidFill>
+                <a:noFill/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>

</xml_diff>

<commit_message>
dodano pierwsza wersje zadania 9
</commit_message>
<xml_diff>
--- a/zadanie_8/wyniki_z_wykresami.xlsx
+++ b/zadanie_8/wyniki_z_wykresami.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kołchoz\Algorytmy\Zadania\zadanie_8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C052D427-07C9-4F23-81B6-020A94446E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F6B68F2-74E3-4F9C-B60B-1D98334060CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{90626785-64BE-41CA-9FCD-EDCBB815A823}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2109" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2111" uniqueCount="14">
   <si>
     <t>Dataset</t>
   </si>
@@ -59,6 +59,12 @@
   </si>
   <si>
     <t>Task2_Peeling</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">   </t>
   </si>
 </sst>
 </file>
@@ -8100,7 +8106,9 @@
             <c:symbol val="circle"/>
             <c:size val="5"/>
             <c:spPr>
-              <a:noFill/>
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
               <a:ln w="9525">
                 <a:noFill/>
               </a:ln>
@@ -9874,10 +9882,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FA0F739-DA7A-4D10-80DB-584C74D07D3D}">
-  <dimension ref="A1:I2101"/>
+  <dimension ref="A1:W2101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -9906,7 +9914,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -9935,7 +9943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -9964,7 +9972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -9993,7 +10001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -10022,7 +10030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -10051,7 +10059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -10080,7 +10088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -10109,7 +10117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -10137,8 +10145,11 @@
       <c r="I9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="W9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -10167,7 +10178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -10196,7 +10207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -10225,7 +10236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -10254,7 +10265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -10283,7 +10294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -10311,8 +10322,11 @@
       <c r="I15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="W15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>9</v>
       </c>

</xml_diff>